<commit_message>
Teklif şablonlarına adet sütunu, Kaan Elektrik şablonu eklendi
Tutar = adet × birim fiyat; ara toplam, %20 KDV ve genel toplam
tutar sütunundan hesaplanır. Kaan Elektrik için aynı yapıda, kendi
logosu ve rengiyle ayrı şablon.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EQEYJfDuBv3YycCTqCV84T
</commit_message>
<xml_diff>
--- a/alker-teklif/Alker_Fiyat_Teklifi.xlsx
+++ b/alker-teklif/Alker_Fiyat_Teklifi.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Teklif" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Teklif!$A$1:$C$44</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Teklif!$A$1:$E$44</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -40,7 +40,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C34" authorId="0">
+    <comment ref="E34" authorId="0">
       <text>
         <r>
           <rPr>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t xml:space="preserve">ALKER YAZILIM</t>
   </si>
@@ -80,7 +80,7 @@
     <t xml:space="preserve">Örnek Firma A.Ş.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Müşteri, tarih, konu ve teklif numarasını üstteki alanlara yazın (B7, C7, B9, C9).</t>
+    <t xml:space="preserve">1. Müşteri, tarih, konu ve teklif numarasını üstteki alanlara yazın (B7, E7, B9, E9).</t>
   </si>
   <si>
     <t xml:space="preserve">KONU</t>
@@ -89,7 +89,7 @@
     <t xml:space="preserve">TEKLİF NO</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Ürünleri B12:B31, fiyatları C12:C31 hücrelerine yazın.</t>
+    <t xml:space="preserve">2. Ürünü B, adedi C, birim fiyatı D sütununa yazın (satır 12–31).</t>
   </si>
   <si>
     <t xml:space="preserve">Kurumsal web sitesi projesi</t>
@@ -98,7 +98,7 @@
     <t xml:space="preserve">ALK-2026-001</t>
   </si>
   <si>
-    <t xml:space="preserve">   Sıra numarası, ürün yazınca kendiliğinden gelir.</t>
+    <t xml:space="preserve">   Tutar (adet × birim fiyat) ve sıra numarası kendiliğinden gelir.</t>
   </si>
   <si>
     <t xml:space="preserve">3. 12. satırdaki örnek ürünü silip kendi ürününüzü yazın.</t>
@@ -110,7 +110,13 @@
     <t xml:space="preserve">Ürün / Hizmet</t>
   </si>
   <si>
-    <t xml:space="preserve">Fiyat (₺)</t>
+    <t xml:space="preserve">Adet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Birim Fiyat (₺)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tutar (₺)</t>
   </si>
   <si>
     <t xml:space="preserve">4. Ara toplam, %20 KDV ve genel toplam otomatik hesaplanır.</t>
@@ -119,7 +125,7 @@
     <t xml:space="preserve">Kurumsal web sitesi (tasarım + yazılım)</t>
   </si>
   <si>
-    <t xml:space="preserve">   KDV oranını değiştirmek için C34 hücresini düzenleyin.</t>
+    <t xml:space="preserve">   KDV oranını değiştirmek için E34 hücresini düzenleyin.</t>
   </si>
   <si>
     <t xml:space="preserve">5. Notları ihtiyaca göre düzenleyin.</t>
@@ -254,6 +260,14 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF141515"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF60646A"/>
       <name val="Arial"/>
@@ -264,14 +278,6 @@
       <b val="true"/>
       <sz val="12"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF141515"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -361,7 +367,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -426,10 +432,18 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -442,27 +456,31 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -764,21 +782,23 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="62"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
@@ -792,15 +812,17 @@
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="G6" s="7" t="s">
         <v>5</v>
       </c>
     </row>
@@ -808,10 +830,10 @@
       <c r="B7" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="E7" s="9" t="n">
         <v>46315</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -819,10 +841,10 @@
       <c r="B8" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>10</v>
       </c>
     </row>
@@ -830,15 +852,15 @@
       <c r="B9" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="E9" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>14</v>
       </c>
     </row>
@@ -849,11 +871,17 @@
       <c r="B11" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="D11" s="13" t="s">
         <v>18</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -862,24 +890,36 @@
         <v>1</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C12" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="17" t="n">
         <v>45000</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>20</v>
+      <c r="E12" s="18" t="n">
+        <f aca="false">IF(OR(C12="",D12=""),"",C12*D12)</f>
+        <v>45000</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17" t="str">
+      <c r="A13" s="19" t="str">
         <f aca="false">IF(B13="","",ROW()-11)</f>
         <v/>
       </c>
-      <c r="B13" s="18"/>
+      <c r="B13" s="20"/>
       <c r="C13" s="19"/>
-      <c r="E13" s="3" t="s">
-        <v>21</v>
+      <c r="D13" s="21"/>
+      <c r="E13" s="22" t="str">
+        <f aca="false">IF(OR(C13="",D13=""),"",C13*D13)</f>
+        <v/>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -889,17 +929,27 @@
       </c>
       <c r="B14" s="15"/>
       <c r="C14" s="16"/>
-      <c r="E14" s="3" t="s">
-        <v>22</v>
+      <c r="D14" s="17"/>
+      <c r="E14" s="18" t="str">
+        <f aca="false">IF(OR(C14="",D14=""),"",C14*D14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17" t="str">
+      <c r="A15" s="19" t="str">
         <f aca="false">IF(B15="","",ROW()-11)</f>
         <v/>
       </c>
-      <c r="B15" s="18"/>
+      <c r="B15" s="20"/>
       <c r="C15" s="19"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="22" t="str">
+        <f aca="false">IF(OR(C15="",D15=""),"",C15*D15)</f>
+        <v/>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="str">
@@ -908,14 +958,24 @@
       </c>
       <c r="B16" s="15"/>
       <c r="C16" s="16"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="18" t="str">
+        <f aca="false">IF(OR(C16="",D16=""),"",C16*D16)</f>
+        <v/>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="str">
+      <c r="A17" s="19" t="str">
         <f aca="false">IF(B17="","",ROW()-11)</f>
         <v/>
       </c>
-      <c r="B17" s="18"/>
+      <c r="B17" s="20"/>
       <c r="C17" s="19"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="22" t="str">
+        <f aca="false">IF(OR(C17="",D17=""),"",C17*D17)</f>
+        <v/>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="str">
@@ -924,14 +984,24 @@
       </c>
       <c r="B18" s="15"/>
       <c r="C18" s="16"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="18" t="str">
+        <f aca="false">IF(OR(C18="",D18=""),"",C18*D18)</f>
+        <v/>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17" t="str">
+      <c r="A19" s="19" t="str">
         <f aca="false">IF(B19="","",ROW()-11)</f>
         <v/>
       </c>
-      <c r="B19" s="18"/>
+      <c r="B19" s="20"/>
       <c r="C19" s="19"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="22" t="str">
+        <f aca="false">IF(OR(C19="",D19=""),"",C19*D19)</f>
+        <v/>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="str">
@@ -940,14 +1010,24 @@
       </c>
       <c r="B20" s="15"/>
       <c r="C20" s="16"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="18" t="str">
+        <f aca="false">IF(OR(C20="",D20=""),"",C20*D20)</f>
+        <v/>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17" t="str">
+      <c r="A21" s="19" t="str">
         <f aca="false">IF(B21="","",ROW()-11)</f>
         <v/>
       </c>
-      <c r="B21" s="18"/>
+      <c r="B21" s="20"/>
       <c r="C21" s="19"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="22" t="str">
+        <f aca="false">IF(OR(C21="",D21=""),"",C21*D21)</f>
+        <v/>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="str">
@@ -956,14 +1036,24 @@
       </c>
       <c r="B22" s="15"/>
       <c r="C22" s="16"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="18" t="str">
+        <f aca="false">IF(OR(C22="",D22=""),"",C22*D22)</f>
+        <v/>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17" t="str">
+      <c r="A23" s="19" t="str">
         <f aca="false">IF(B23="","",ROW()-11)</f>
         <v/>
       </c>
-      <c r="B23" s="18"/>
+      <c r="B23" s="20"/>
       <c r="C23" s="19"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="22" t="str">
+        <f aca="false">IF(OR(C23="",D23=""),"",C23*D23)</f>
+        <v/>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="str">
@@ -972,14 +1062,24 @@
       </c>
       <c r="B24" s="15"/>
       <c r="C24" s="16"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="18" t="str">
+        <f aca="false">IF(OR(C24="",D24=""),"",C24*D24)</f>
+        <v/>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17" t="str">
+      <c r="A25" s="19" t="str">
         <f aca="false">IF(B25="","",ROW()-11)</f>
         <v/>
       </c>
-      <c r="B25" s="18"/>
+      <c r="B25" s="20"/>
       <c r="C25" s="19"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="22" t="str">
+        <f aca="false">IF(OR(C25="",D25=""),"",C25*D25)</f>
+        <v/>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="str">
@@ -988,14 +1088,24 @@
       </c>
       <c r="B26" s="15"/>
       <c r="C26" s="16"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="18" t="str">
+        <f aca="false">IF(OR(C26="",D26=""),"",C26*D26)</f>
+        <v/>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17" t="str">
+      <c r="A27" s="19" t="str">
         <f aca="false">IF(B27="","",ROW()-11)</f>
         <v/>
       </c>
-      <c r="B27" s="18"/>
+      <c r="B27" s="20"/>
       <c r="C27" s="19"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="22" t="str">
+        <f aca="false">IF(OR(C27="",D27=""),"",C27*D27)</f>
+        <v/>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="str">
@@ -1004,14 +1114,24 @@
       </c>
       <c r="B28" s="15"/>
       <c r="C28" s="16"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="18" t="str">
+        <f aca="false">IF(OR(C28="",D28=""),"",C28*D28)</f>
+        <v/>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="17" t="str">
+      <c r="A29" s="19" t="str">
         <f aca="false">IF(B29="","",ROW()-11)</f>
         <v/>
       </c>
-      <c r="B29" s="18"/>
+      <c r="B29" s="20"/>
       <c r="C29" s="19"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="22" t="str">
+        <f aca="false">IF(OR(C29="",D29=""),"",C29*D29)</f>
+        <v/>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="14" t="str">
@@ -1020,83 +1140,102 @@
       </c>
       <c r="B30" s="15"/>
       <c r="C30" s="16"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="18" t="str">
+        <f aca="false">IF(OR(C30="",D30=""),"",C30*D30)</f>
+        <v/>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="17" t="str">
+      <c r="A31" s="19" t="str">
         <f aca="false">IF(B31="","",ROW()-11)</f>
         <v/>
       </c>
-      <c r="B31" s="18"/>
+      <c r="B31" s="20"/>
       <c r="C31" s="19"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="22" t="str">
+        <f aca="false">IF(OR(C31="",D31=""),"",C31*D31)</f>
+        <v/>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="C33" s="21" t="n">
-        <f aca="false">SUM(C12:C31)</f>
+      <c r="D33" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="E33" s="24" t="n">
+        <f aca="false">SUM(E12:E31)</f>
         <v>45000</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="20" t="s">
-        <v>24</v>
-      </c>
-      <c r="C34" s="22" t="n">
+      <c r="D34" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="E34" s="25" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="20" t="s">
-        <v>25</v>
-      </c>
-      <c r="C35" s="21" t="n">
-        <f aca="false">C33*C34</f>
+      <c r="D35" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="E35" s="24" t="n">
+        <f aca="false">E33*E34</f>
         <v>9000</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="C36" s="24" t="n">
-        <f aca="false">C33+C35</f>
+      <c r="B36" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="C36" s="26"/>
+      <c r="D36" s="26"/>
+      <c r="E36" s="27" t="n">
+        <f aca="false">E33+E35</f>
         <v>54000</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C43" s="25" t="s">
-        <v>31</v>
+      <c r="E43" s="28" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C44" s="26" t="s">
-        <v>32</v>
+      <c r="E44" s="29" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation allowBlank="false" error="Fiyat 0 veya daha büyük bir sayı olmalı." errorStyle="stop" errorTitle="Geçersiz fiyat" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C12:C31" type="decimal">
+  <mergeCells count="1">
+    <mergeCell ref="B36:D36"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation allowBlank="false" error="Adet 0'dan büyük bir sayı olmalı." errorStyle="stop" errorTitle="Geçersiz adet" operator="greaterThan" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C12:C31" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="Fiyat 0 veya daha büyük bir sayı olmalı." errorStyle="stop" errorTitle="Geçersiz fiyat" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D12:D31" type="decimal">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>